<commit_message>
Batch 2 (S2) results: 114 verified rules for 89 entries; sibling-page families kept as links
- Full run over the 267 path entries of batch 2: static crawl, sitemaps, rendering,
  hash-route click sampling (Kuaishou, Alimama, incoPat) with browser identity checks
- Families whose only false match is the entry page itself are the entry's sibling
  pages (e.g. other channels next to /lists/2.html), not its children: kept as links
  instead of reported as failed (batch 1: Census and ITU move the same way)
- Hash-route rules merged into the ledger and result table; entries without a scheme
  note the scheme that was actually verified
- export_patterns.py writes patterns-final.xlsx|csv for any batch
- Raw crawl data committed gzip-compressed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HW9kjaADHDgTyps9HbQ9Ce
</commit_message>
<xml_diff>
--- a/url-pattern-verification/output/round3/patterns-final.xlsx
+++ b/url-pattern-verification/output/round3/patterns-final.xlsx
@@ -6054,7 +6054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6111,61 +6111,61 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>S1-R2-E1</t>
+          <t>S1-R18-E4</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.census.gov/retail/</t>
+          <t>https://www.itu.int/en/action/Pages/default.aspx</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.census\.gov/retail/[a-z_]+\.html$</t>
+          <t>^https://www\.itu\.int/en/action/[a-z-]+/Pages/default\.aspx$</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>验证不通过</t>
+          <t>部分验证（候选）</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.census.gov/retail/definitions.html</t>
+          <t>https://www.itu.int/en/action/gender-equality/Pages/default.aspx</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R2-E1-F1</t>
+          <t>R3-S1-R18-E4-F2</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：归纳正例 2&lt;3、标注测试有失败（留出 FN0/FP1）、留出指标 &lt;95%</t>
+          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>S1-R18-E4</t>
+          <t>S1-R19-E12</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://www.itu.int/en/action/Pages/default.aspx</t>
+          <t>https://www.wipo.int/en/web/business</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.itu\.int/en/action/[a-z-]+/Pages/default\.aspx$</t>
+          <t>^https://www\.wipo\.int/en/web/business/[a-z-]+$</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -6175,77 +6175,77 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.itu.int/en/action/gender-equality/Pages/default.aspx</t>
+          <t>https://www.wipo.int/en/web/business/checklist</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R18-E4-F2</t>
+          <t>R3-S1-R19-E12-F1</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
+          <t>机械门未通过：留出与归纳/回归重叠；列表成员漏配 1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>S1-R18-E7</t>
+          <t>S1-R19-E4</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.itu.int/en/ITU-D/Pages/default.aspx</t>
+          <t>https://www.wipo.int/en/web/patentscope/</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.itu\.int/en/ITU\-D/Pages/[a-zA-Z0-9-]+\.aspx$</t>
+          <t>^https://www\.wipo\.int/en/web/patentscope/[a-z_]+$</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>验证不通过</t>
+          <t>部分验证（候选）</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.itu.int/en/ITU-D/Pages/ITUAroundTheWorld.aspx</t>
+          <t>https://www.wipo.int/en/web/patentscope/national_databases</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R18-E7-F1</t>
+          <t>R3-S1-R19-E4-F1</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：标注测试有失败（留出 FN0/FP1）、留出指标 &lt;95%</t>
+          <t>机械门未通过：归纳正例 2&lt;3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>S1-R19-E12</t>
+          <t>S1-R27-E1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/en/web/business</t>
+          <t>https://www.euromonitor.com/articles</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.wipo\.int/en/web/business/[a-z-]+$</t>
+          <t>^https://www\.euromonitor\.com/insights/insight\-search\-result\-page\-tags\?tag=[a-zA-Z_-]*&amp;returnUrl=[a-zA-Z0-9%\.]*$</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -6255,37 +6255,37 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/en/web/business/checklist</t>
+          <t>https://www.euromonitor.com/insights/insight-search-result-page-tags?tag=Apparel-and-Footwear&amp;returnUrl=https%3A%2F%2Fwww.euromonitor.com%2Fwebinar%3Famp</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R19-E12-F1</t>
+          <t>R3-S1-R27-E1-F2</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：留出与归纳/回归重叠；列表成员漏配 1</t>
+          <t>机械门未通过：留出与归纳/回归重叠</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>S1-R19-E4</t>
+          <t>S1-R35-E1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/en/web/patentscope/</t>
+          <t>https://www.comscore.com/Insights/Blog</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.wipo\.int/en/web/patentscope/[a-z_]+$</t>
+          <t>^https://www\.comscore\.com/Insights/Blog/[a-zA-Z0-9-]+$</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -6295,37 +6295,37 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/en/web/patentscope/national_databases</t>
+          <t>https://www.comscore.com/Insights/Blog/Consumer-AI-Chatbots-Keep-Climbing-in-March</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R19-E4-F1</t>
+          <t>R3-S1-R35-E1-F1</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：归纳正例 2&lt;3</t>
+          <t>机械门未通过：留出与归纳/回归重叠</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>27</v>
+        <v>86</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>S1-R27-E1</t>
+          <t>S1-R86-E1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://www.euromonitor.com/articles</t>
+          <t>https://www.dandad.org/work/annual-2026/</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.euromonitor\.com/insights/insight\-search\-result\-page\-tags\?tag=[a-zA-Z_-]*&amp;returnUrl=[a-zA-Z0-9%\.]*$</t>
+          <t>^https://www\.dandad\.org/work/annual\-2026/[a-z0-9-]+$</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -6335,37 +6335,37 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://www.euromonitor.com/insights/insight-search-result-page-tags?tag=Apparel-and-Footwear&amp;returnUrl=https%3A%2F%2Fwww.euromonitor.com%2Fwebinar%3Famp</t>
+          <t>https://www.dandad.org/work/annual-2026/behind-the-work</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R27-E1-F2</t>
+          <t>R3-S1-R86-E1-F2</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：留出与归纳/回归重叠</t>
+          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>S1-R35-E1</t>
+          <t>S1-R91-E1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.comscore.com/Insights/Blog</t>
+          <t>https://growthhackers.com/growth-studies/</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.comscore\.com/Insights/Blog/[a-zA-Z0-9-]+$</t>
+          <t>^https://growthhackers\.com/growth\-studies/[a-z-]+/$</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -6375,37 +6375,37 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.comscore.com/Insights/Blog/Consumer-AI-Chatbots-Keep-Climbing-in-March</t>
+          <t>https://growthhackers.com/growth-studies/uber/</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R35-E1-F1</t>
+          <t>R3-S1-R91-E1-F1</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>机械门未通过：留出与归纳/回归重叠</t>
+          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>86</v>
+        <v>133</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>S1-R86-E1</t>
+          <t>S1-R133-E1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://www.dandad.org/work/annual-2026/</t>
+          <t>https://www.siegelgale.com/ideas/</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>^https://www\.dandad\.org/work/annual\-2026/[a-z0-9-]+$</t>
+          <t>^https://www\.siegelgale\.com/ideas/[a-z-]+/$</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -6415,95 +6415,15 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://www.dandad.org/work/annual-2026/behind-the-work</t>
+          <t>https://www.siegelgale.com/ideas/ai/</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>R3-S1-R86-E1-F2</t>
+          <t>R3-S1-R133-E1-F1</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>S1-R91-E1</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>https://growthhackers.com/growth-studies/</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>^https://growthhackers\.com/growth\-studies/[a-z-]+/$</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>部分验证（候选）</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>https://growthhackers.com/growth-studies/uber/</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>R3-S1-R91-E1-F1</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>133</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>S1-R133-E1</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.siegelgale.com/ideas/</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>^https://www\.siegelgale\.com/ideas/[a-z-]+/$</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>部分验证（候选）</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.siegelgale.com/ideas/ai/</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>R3-S1-R133-E1-F1</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）</t>
         </is>

</xml_diff>